<commit_message>
feat: update test data file with percentage values and outlier
</commit_message>
<xml_diff>
--- a/data/test/testData_with_perc.xlsx
+++ b/data/test/testData_with_perc.xlsx
@@ -1,23 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meissnerto\Desktop\texAn.R\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meissnerto\Desktop\TexAn2.0\data\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B06297A3-1147-46F5-9E41-845BDB18AD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20925" windowHeight="17820"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -188,7 +203,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.00000000"/>
@@ -598,7 +613,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -673,11 +688,11 @@
       </c>
       <c r="K2" s="7">
         <f ca="1">RANDBETWEEN(70,99)/100</f>
-        <v>0.73</v>
+        <v>0.82</v>
       </c>
       <c r="L2" s="15">
         <f ca="1">RANDBETWEEN(70,99)</f>
-        <v>99</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -713,11 +728,11 @@
       </c>
       <c r="K3" s="7">
         <f t="shared" ref="K3:K66" ca="1" si="0">RANDBETWEEN(70,99)/100</f>
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L3" s="15">
         <f t="shared" ref="L3:L66" ca="1" si="1">RANDBETWEEN(70,99)</f>
-        <v>93</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -753,11 +768,11 @@
       </c>
       <c r="K4" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.78</v>
+        <v>0.94</v>
       </c>
       <c r="L4" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -793,11 +808,11 @@
       </c>
       <c r="K5" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.86</v>
+        <v>0.77</v>
       </c>
       <c r="L5" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -833,11 +848,11 @@
       </c>
       <c r="K6" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.87</v>
+        <v>0.94</v>
       </c>
       <c r="L6" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -873,11 +888,11 @@
       </c>
       <c r="K7" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="L7" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -913,11 +928,11 @@
       </c>
       <c r="K8" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="L8" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -953,11 +968,11 @@
       </c>
       <c r="K9" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.81</v>
+        <v>0.8</v>
       </c>
       <c r="L9" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -993,11 +1008,11 @@
       </c>
       <c r="K10" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="L10" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1033,11 +1048,11 @@
       </c>
       <c r="K11" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.89</v>
+        <v>0.81</v>
       </c>
       <c r="L11" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>90</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1063,7 +1078,7 @@
         <v>2</v>
       </c>
       <c r="H12" s="14">
-        <v>0.81757800541450043</v>
+        <v>3</v>
       </c>
       <c r="I12">
         <v>90.352346559462731</v>
@@ -1073,11 +1088,11 @@
       </c>
       <c r="K12" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.74</v>
+        <v>0.8</v>
       </c>
       <c r="L12" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>70</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1113,11 +1128,11 @@
       </c>
       <c r="K13" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.77</v>
+        <v>0.97</v>
       </c>
       <c r="L13" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1153,11 +1168,11 @@
       </c>
       <c r="K14" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.71</v>
       </c>
       <c r="L14" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1193,11 +1208,11 @@
       </c>
       <c r="K15" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
       <c r="L15" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -1233,11 +1248,11 @@
       </c>
       <c r="K16" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="L16" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -1277,7 +1292,7 @@
       </c>
       <c r="L17" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1313,11 +1328,11 @@
       </c>
       <c r="K18" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="L18" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -1353,11 +1368,11 @@
       </c>
       <c r="K19" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.81</v>
       </c>
       <c r="L19" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -1393,11 +1408,11 @@
       </c>
       <c r="K20" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
       <c r="L20" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>70</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -1433,11 +1448,11 @@
       </c>
       <c r="K21" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.78</v>
+        <v>0.92</v>
       </c>
       <c r="L21" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>95</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -1473,11 +1488,11 @@
       </c>
       <c r="K22" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.76</v>
       </c>
       <c r="L22" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>86</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
@@ -1513,11 +1528,11 @@
       </c>
       <c r="K23" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
       <c r="L23" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -1553,11 +1568,11 @@
       </c>
       <c r="K24" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.75</v>
+        <v>0.82</v>
       </c>
       <c r="L24" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -1593,11 +1608,11 @@
       </c>
       <c r="K25" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.97</v>
+        <v>0.75</v>
       </c>
       <c r="L25" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>89</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -1633,11 +1648,11 @@
       </c>
       <c r="K26" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.83</v>
+        <v>0.94</v>
       </c>
       <c r="L26" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>80</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
@@ -1673,11 +1688,11 @@
       </c>
       <c r="K27" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.76</v>
       </c>
       <c r="L27" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -1713,11 +1728,11 @@
       </c>
       <c r="K28" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="L28" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -1753,11 +1768,11 @@
       </c>
       <c r="K29" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.94</v>
+        <v>0.82</v>
       </c>
       <c r="L29" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>89</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -1793,11 +1808,11 @@
       </c>
       <c r="K30" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.93</v>
+        <v>0.81</v>
       </c>
       <c r="L30" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -1833,11 +1848,11 @@
       </c>
       <c r="K31" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.85</v>
+        <v>0.79</v>
       </c>
       <c r="L31" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>97</v>
+        <v>85</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
@@ -1873,11 +1888,11 @@
       </c>
       <c r="K32" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="L32" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>76</v>
+        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
@@ -1913,11 +1928,11 @@
       </c>
       <c r="K33" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.79</v>
+        <v>0.99</v>
       </c>
       <c r="L33" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
@@ -1953,11 +1968,11 @@
       </c>
       <c r="K34" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.73</v>
+        <v>0.99</v>
       </c>
       <c r="L34" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
@@ -1993,11 +2008,11 @@
       </c>
       <c r="K35" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.72</v>
+        <v>0.81</v>
       </c>
       <c r="L35" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
@@ -2033,11 +2048,11 @@
       </c>
       <c r="K36" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="L36" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>94</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
@@ -2073,11 +2088,11 @@
       </c>
       <c r="K37" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.98</v>
+        <v>0.94</v>
       </c>
       <c r="L37" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
@@ -2113,11 +2128,11 @@
       </c>
       <c r="K38" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.75</v>
+        <v>0.83</v>
       </c>
       <c r="L38" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>74</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
@@ -2153,11 +2168,11 @@
       </c>
       <c r="K39" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="L39" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
@@ -2193,11 +2208,11 @@
       </c>
       <c r="K40" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.86</v>
+        <v>0.96</v>
       </c>
       <c r="L40" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -2233,11 +2248,11 @@
       </c>
       <c r="K41" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.98</v>
+        <v>0.85</v>
       </c>
       <c r="L41" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>75</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
@@ -2273,11 +2288,11 @@
       </c>
       <c r="K42" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.77</v>
+        <v>0.99</v>
       </c>
       <c r="L42" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>96</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
@@ -2313,11 +2328,11 @@
       </c>
       <c r="K43" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.71</v>
+        <v>0.87</v>
       </c>
       <c r="L43" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>88</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -2353,11 +2368,11 @@
       </c>
       <c r="K44" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.82</v>
+        <v>0.9</v>
       </c>
       <c r="L44" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -2393,11 +2408,11 @@
       </c>
       <c r="K45" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="L45" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>89</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
@@ -2433,11 +2448,11 @@
       </c>
       <c r="K46" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.77</v>
+        <v>0.89</v>
       </c>
       <c r="L46" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
@@ -2473,11 +2488,11 @@
       </c>
       <c r="K47" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.95</v>
+        <v>0.77</v>
       </c>
       <c r="L47" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>71</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
@@ -2513,11 +2528,11 @@
       </c>
       <c r="K48" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.76</v>
+        <v>0.81</v>
       </c>
       <c r="L48" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
@@ -2557,7 +2572,7 @@
       </c>
       <c r="L49" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
@@ -2593,11 +2608,11 @@
       </c>
       <c r="K50" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="L50" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>84</v>
+        <v>72</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
@@ -2633,11 +2648,11 @@
       </c>
       <c r="K51" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="L51" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
@@ -2673,11 +2688,11 @@
       </c>
       <c r="K52" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.91</v>
+        <v>0.9</v>
       </c>
       <c r="L52" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
@@ -2713,11 +2728,11 @@
       </c>
       <c r="K53" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.73</v>
+        <v>0.99</v>
       </c>
       <c r="L53" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
@@ -2753,11 +2768,11 @@
       </c>
       <c r="K54" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.73</v>
+        <v>0.95</v>
       </c>
       <c r="L54" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
@@ -2793,11 +2808,11 @@
       </c>
       <c r="K55" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="L55" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>99</v>
+        <v>78</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
@@ -2833,11 +2848,11 @@
       </c>
       <c r="K56" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="L56" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>85</v>
+        <v>71</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
@@ -2873,11 +2888,11 @@
       </c>
       <c r="K57" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="L57" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>89</v>
+        <v>75</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
@@ -2913,11 +2928,11 @@
       </c>
       <c r="K58" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.76</v>
+        <v>0.98</v>
       </c>
       <c r="L58" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>99</v>
+        <v>86</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
@@ -2943,7 +2958,7 @@
         <v>1</v>
       </c>
       <c r="H59">
-        <v>3.548867167204889</v>
+        <v>-2</v>
       </c>
       <c r="I59">
         <v>96.414966601406064</v>
@@ -2953,11 +2968,11 @@
       </c>
       <c r="K59" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.76</v>
+        <v>0.71</v>
       </c>
       <c r="L59" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
@@ -2993,11 +3008,11 @@
       </c>
       <c r="K60" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.96</v>
+        <v>0.71</v>
       </c>
       <c r="L60" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
@@ -3033,11 +3048,11 @@
       </c>
       <c r="K61" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L61" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
@@ -3073,11 +3088,11 @@
       </c>
       <c r="K62" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L62" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>75</v>
+        <v>83</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
@@ -3117,7 +3132,7 @@
       </c>
       <c r="L63" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>85</v>
+        <v>71</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -3153,11 +3168,11 @@
       </c>
       <c r="K64" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="L64" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
@@ -3193,11 +3208,11 @@
       </c>
       <c r="K65" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.8</v>
+        <v>0.88</v>
       </c>
       <c r="L65" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
@@ -3233,11 +3248,11 @@
       </c>
       <c r="K66" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0.74</v>
+        <v>0.94</v>
       </c>
       <c r="L66" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>87</v>
+        <v>98</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
@@ -3273,11 +3288,11 @@
       </c>
       <c r="K67" s="7">
         <f t="shared" ref="K67:K73" ca="1" si="2">RANDBETWEEN(70,99)/100</f>
-        <v>0.96</v>
+        <v>0.73</v>
       </c>
       <c r="L67" s="15">
         <f t="shared" ref="L67:L73" ca="1" si="3">RANDBETWEEN(70,99)</f>
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
@@ -3313,11 +3328,11 @@
       </c>
       <c r="K68" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>0.87</v>
+        <v>0.77</v>
       </c>
       <c r="L68" s="15">
         <f t="shared" ca="1" si="3"/>
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
@@ -3353,11 +3368,11 @@
       </c>
       <c r="K69" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="L69" s="15">
         <f t="shared" ca="1" si="3"/>
-        <v>74</v>
+        <v>90</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
@@ -3393,11 +3408,11 @@
       </c>
       <c r="K70" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>0.79</v>
+        <v>0.98</v>
       </c>
       <c r="L70" s="15">
         <f t="shared" ca="1" si="3"/>
-        <v>80</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
@@ -3433,11 +3448,11 @@
       </c>
       <c r="K71" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>0.85</v>
+        <v>0.71</v>
       </c>
       <c r="L71" s="15">
         <f t="shared" ca="1" si="3"/>
-        <v>99</v>
+        <v>83</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
@@ -3473,11 +3488,11 @@
       </c>
       <c r="K72" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>0.77</v>
+        <v>0.72</v>
       </c>
       <c r="L72" s="15">
         <f t="shared" ca="1" si="3"/>
-        <v>93</v>
+        <v>76</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
@@ -3513,11 +3528,11 @@
       </c>
       <c r="K73" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>0.97</v>
+        <v>0.78</v>
       </c>
       <c r="L73" s="15">
         <f t="shared" ca="1" si="3"/>
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>